<commit_message>
Push outputs from CI/CD (2026-10-13 19:09:34)
</commit_message>
<xml_diff>
--- a/production/watch-CHECKED/Manufacturing/Assembly/ZSWatch-Watch-bom.xlsx
+++ b/production/watch-CHECKED/Manufacturing/Assembly/ZSWatch-Watch-bom.xlsx
@@ -1061,10 +1061,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-02-20 19:32:44</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.5</t>
+    <t>2026-10-13 19:16:05</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.21 + KiBot v1.9.1</t>
   </si>
   <si>
     <t>Columns colors</t>
@@ -4332,7 +4332,7 @@
     <row r="87" spans="10:10" ht="30" hidden="1" customHeight="1">
       <c r="J87" t="str">
         <f t="array" ref="J87:J123">IF(ISNUMBER(J10:J46)*(J10:J46&gt;=L10:L46)*(N10:N46&lt;&gt;""),N10:N46&amp;"|"&amp;TEXT(ROUNDUP(J10:J46/IF(ISNUMBER(L10:L46),L10:L46,1),0)*L10:L46,"##0")&amp;"|"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(PURCHASE_DESCRIPTION&lt;&gt;"",PURCHASE_DESCRIPTION&amp;":","")&amp;A10:A46,"|",";")," ","_"),"
-","_")&amp;CHAR(10),"")</f>
+","_")&amp;CHAR(13),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>